<commit_message>
Add: created and tested PolygonCalculator.setPerimeter, .setCorrectrionsHorAngle
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="PotenotTask test data" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="InverseTask test data" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Survey test data" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Polygon test data" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="138">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -365,6 +366,78 @@
   </si>
   <si>
     <t xml:space="preserve">targets for 101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horAngle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">correctionHorAngle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">directionAngle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">corrX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">corrY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">456961.430</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261163.707</t>
+  </si>
+  <si>
+    <t xml:space="preserve">456988.790</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261202.196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">457057.453</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261204.245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">457122.419</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261202.416</t>
+  </si>
+  <si>
+    <t xml:space="preserve">457129.441</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261145.698</t>
+  </si>
+  <si>
+    <t xml:space="preserve">457129.609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261111.97</t>
+  </si>
+  <si>
+    <t xml:space="preserve">457131.018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2261065.036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">∑ = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fhor = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CorrHor =</t>
   </si>
 </sst>
 </file>
@@ -379,7 +452,7 @@
     <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="169" formatCode="[hh]:mm:ss"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -467,6 +540,12 @@
       <color rgb="FF800080"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -562,7 +641,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -691,6 +770,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -769,7 +852,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.15625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1365,7 +1448,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.07421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2450,7 +2533,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2620,7 +2703,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3219,4 +3302,301 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.16"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="H1" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="I1" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K1" s="29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="n">
+        <v>196534</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>457619</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>653188</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>978190</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <f aca="false">SUM(B3:B7)</f>
+        <v>2725711</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add: created and tested PolygonCalculator.setDirectionAngle by direct order
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -452,7 +452,7 @@
     <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="169" formatCode="[hh]:mm:ss"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -538,6 +538,13 @@
       <i val="true"/>
       <sz val="10"/>
       <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00A933"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -641,7 +648,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -774,6 +781,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -852,7 +863,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.15625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.19140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1448,7 +1459,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2533,7 +2544,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2703,7 +2714,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3310,10 +3321,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.16"/>
   </cols>
@@ -3364,7 +3375,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="1"/>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="32" t="n">
         <v>196534</v>
       </c>
       <c r="F2" s="1"/>
@@ -3390,7 +3401,9 @@
       <c r="D3" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="1" t="n">
+        <v>6142</v>
+      </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -3414,7 +3427,9 @@
       <c r="D4" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E4" s="1"/>
+      <c r="E4" s="1" t="n">
+        <v>1290184</v>
+      </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -3438,7 +3453,9 @@
       <c r="D5" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E5" s="1"/>
+      <c r="E5" s="1" t="n">
+        <v>997390</v>
+      </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -3462,7 +3479,9 @@
       <c r="D6" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E6" s="1"/>
+      <c r="E6" s="1" t="n">
+        <v>973013</v>
+      </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -3486,7 +3505,7 @@
       <c r="D7" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="32" t="n">
         <v>978190</v>
       </c>
       <c r="F7" s="1"/>
@@ -3536,7 +3555,7 @@
       <c r="L9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="33" t="s">
         <v>135</v>
       </c>
       <c r="B10" s="1" t="n">

</xml_diff>

<commit_message>
Add: PolygonCalculator.doubleToLong, .doubleToLongTest, setDeltaXY, setDeltaXYTest  setCorrectionXY, setCorrectionTestResiduals
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -389,48 +389,6 @@
     <t xml:space="preserve">corrY</t>
   </si>
   <si>
-    <t xml:space="preserve">456961.430</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261163.707</t>
-  </si>
-  <si>
-    <t xml:space="preserve">456988.790</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261202.196</t>
-  </si>
-  <si>
-    <t xml:space="preserve">457057.453</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261204.245</t>
-  </si>
-  <si>
-    <t xml:space="preserve">457122.419</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261202.416</t>
-  </si>
-  <si>
-    <t xml:space="preserve">457129.441</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261145.698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">457129.609</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261111.97</t>
-  </si>
-  <si>
-    <t xml:space="preserve">457131.018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2261065.036</t>
-  </si>
-  <si>
     <t xml:space="preserve">∑ = </t>
   </si>
   <si>
@@ -438,6 +396,24 @@
   </si>
   <si>
     <t xml:space="preserve">CorrHor =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FX = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perimeter = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabs = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fotn = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:11228</t>
   </si>
 </sst>
 </file>
@@ -863,7 +839,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.19140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1459,7 +1435,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2544,7 +2520,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2714,7 +2690,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3320,13 +3296,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.57"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3374,19 +3354,14 @@
       <c r="C2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="1"/>
       <c r="E2" s="32" t="n">
         <v>196534</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>122</v>
+      <c r="J2" s="32" t="n">
+        <v>456961430</v>
+      </c>
+      <c r="K2" s="32" t="n">
+        <v>2261163707</v>
       </c>
       <c r="L2" s="1"/>
     </row>
@@ -3397,22 +3372,29 @@
       <c r="B3" s="1" t="n">
         <v>457619</v>
       </c>
-      <c r="C3" s="1"/>
       <c r="D3" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>6142</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>124</v>
+      <c r="F3" s="1" t="n">
+        <v>68659</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>2045</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="32" t="n">
+        <v>456988790</v>
+      </c>
+      <c r="K3" s="32" t="n">
+        <v>2261202196</v>
       </c>
       <c r="L3" s="1"/>
     </row>
@@ -3423,22 +3405,29 @@
       <c r="B4" s="1" t="n">
         <v>636053</v>
       </c>
-      <c r="C4" s="1"/>
       <c r="D4" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>1290184</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>126</v>
+      <c r="F4" s="1" t="n">
+        <v>64961</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>-1832</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>457057453</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>2261204245</v>
       </c>
       <c r="L4" s="1"/>
     </row>
@@ -3449,22 +3438,29 @@
       <c r="B5" s="1" t="n">
         <v>355217</v>
       </c>
-      <c r="C5" s="1"/>
       <c r="D5" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>997390</v>
       </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>128</v>
+      <c r="F5" s="1" t="n">
+        <v>7018</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>-56722</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>457122419</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>2261202416</v>
       </c>
       <c r="L5" s="1"/>
     </row>
@@ -3475,22 +3471,29 @@
       <c r="B6" s="1" t="n">
         <v>623634</v>
       </c>
-      <c r="C6" s="1"/>
       <c r="D6" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>973013</v>
       </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>130</v>
+      <c r="F6" s="1" t="n">
+        <v>166</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>-33730</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>457129441</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>2261145698</v>
       </c>
       <c r="L6" s="1"/>
     </row>
@@ -3501,22 +3504,17 @@
       <c r="B7" s="1" t="n">
         <v>653188</v>
       </c>
-      <c r="C7" s="1"/>
       <c r="D7" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E7" s="32" t="n">
         <v>978190</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>132</v>
+      <c r="J7" s="32" t="n">
+        <v>457129609</v>
+      </c>
+      <c r="K7" s="32" t="n">
+        <v>2261111970</v>
       </c>
       <c r="L7" s="1"/>
     </row>
@@ -3524,90 +3522,102 @@
       <c r="A8" s="1" t="n">
         <v>1004</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>134</v>
+      <c r="J8" s="32" t="n">
+        <v>457131018</v>
+      </c>
+      <c r="K8" s="32" t="n">
+        <v>2261065036</v>
       </c>
       <c r="L8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">SUM(B3:B7)</f>
         <v>2725711</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
+      <c r="F10" s="1" t="n">
+        <f aca="false">SUM(F3:F6)</f>
+        <v>140804</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <f aca="false">SUM(H3:H6)</f>
+        <v>-90239</v>
+      </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <f aca="false">J3+F10-J7</f>
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <f aca="false">K3+H10-K7</f>
+        <v>-13</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>224560</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>129</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add: PolygonCalculator.setCorrectionZ, .setXYZ, .setCorrectionZTest, .setXYZTest, .adjustPolygonTestTT
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="134">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -389,6 +389,12 @@
     <t xml:space="preserve">corrY</t>
   </si>
   <si>
+    <t xml:space="preserve">DZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">corrZ</t>
+  </si>
+  <si>
     <t xml:space="preserve">∑ = </t>
   </si>
   <si>
@@ -414,6 +420,12 @@
   </si>
   <si>
     <t xml:space="preserve">1:11228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fh = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RatioZ = </t>
   </si>
 </sst>
 </file>
@@ -839,7 +851,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.2109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1435,7 +1447,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.12109375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2520,7 +2532,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2690,7 +2702,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3296,8 +3308,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:N20"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
@@ -3307,6 +3319,8 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.65"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="21.22"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11.59"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3343,6 +3357,15 @@
       <c r="K1" s="29" t="s">
         <v>108</v>
       </c>
+      <c r="L1" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="N1" s="29" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
@@ -3363,7 +3386,8 @@
       <c r="K2" s="32" t="n">
         <v>2261163707</v>
       </c>
-      <c r="L2" s="1"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -3372,6 +3396,9 @@
       <c r="B3" s="1" t="n">
         <v>457619</v>
       </c>
+      <c r="C3" s="1" t="n">
+        <v>68689</v>
+      </c>
       <c r="D3" s="1" t="n">
         <v>-11</v>
       </c>
@@ -3396,7 +3423,16 @@
       <c r="K3" s="32" t="n">
         <v>2261202196</v>
       </c>
-      <c r="L3" s="1"/>
+      <c r="L3" s="1" t="n">
+        <v>-286</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <f aca="false">C3*B20</f>
+        <v>-1.52941307445672</v>
+      </c>
+      <c r="N3" s="32" t="n">
+        <v>17720</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
@@ -3405,6 +3441,9 @@
       <c r="B4" s="1" t="n">
         <v>636053</v>
       </c>
+      <c r="C4" s="1" t="n">
+        <v>64987</v>
+      </c>
       <c r="D4" s="1" t="n">
         <v>-11</v>
       </c>
@@ -3415,7 +3454,7 @@
         <v>64961</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H4" s="1" t="n">
         <v>-1832</v>
@@ -3429,7 +3468,16 @@
       <c r="K4" s="1" t="n">
         <v>2261204245</v>
       </c>
-      <c r="L4" s="1"/>
+      <c r="L4" s="1" t="n">
+        <v>-174</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <f aca="false">C4*B20</f>
+        <v>-1.4469852155326</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>17429</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
@@ -3438,6 +3486,9 @@
       <c r="B5" s="1" t="n">
         <v>355217</v>
       </c>
+      <c r="C5" s="1" t="n">
+        <v>57154</v>
+      </c>
       <c r="D5" s="1" t="n">
         <v>-11</v>
       </c>
@@ -3462,7 +3513,16 @@
       <c r="K5" s="1" t="n">
         <v>2261202416</v>
       </c>
-      <c r="L5" s="1"/>
+      <c r="L5" s="1" t="n">
+        <v>-928</v>
+      </c>
+      <c r="M5" s="1" t="n">
+        <f aca="false">C5*B20</f>
+        <v>-1.27257748485928</v>
+      </c>
+      <c r="N5" s="1" t="n">
+        <v>17255</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
@@ -3471,6 +3531,9 @@
       <c r="B6" s="1" t="n">
         <v>623634</v>
       </c>
+      <c r="C6" s="1" t="n">
+        <v>33730</v>
+      </c>
       <c r="D6" s="1" t="n">
         <v>-11</v>
       </c>
@@ -3495,7 +3558,16 @@
       <c r="K6" s="1" t="n">
         <v>2261145698</v>
       </c>
-      <c r="L6" s="1"/>
+      <c r="L6" s="1" t="n">
+        <v>-560</v>
+      </c>
+      <c r="M6" s="1" t="n">
+        <f aca="false">C6*B20</f>
+        <v>-0.751024225151407</v>
+      </c>
+      <c r="N6" s="1" t="n">
+        <v>16327</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
@@ -3516,7 +3588,11 @@
       <c r="K7" s="32" t="n">
         <v>2261111970</v>
       </c>
-      <c r="L7" s="1"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32" t="n">
+        <v>15767</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
@@ -3528,16 +3604,18 @@
       <c r="K8" s="32" t="n">
         <v>2261065036</v>
       </c>
-      <c r="L8" s="1"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">SUM(B3:B7)</f>
@@ -3553,11 +3631,15 @@
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
+      <c r="L10" s="1" t="n">
+        <f aca="false">SUM(L3:L6)</f>
+        <v>-1948</v>
+      </c>
+      <c r="M10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>55</v>
@@ -3565,10 +3647,11 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-11</v>
@@ -3576,10 +3659,11 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">J3+F10-J7</f>
@@ -3588,7 +3672,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B14" s="1" t="n">
         <f aca="false">K3+H10-K7</f>
@@ -3597,7 +3681,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>224560</v>
@@ -3605,7 +3689,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>20</v>
@@ -3613,10 +3697,28 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <f aca="false">N3+L10-N7</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <f aca="false">B19/B15*-1</f>
+        <v>-2.2265764161026E-005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add: PolygonCalculator.adjustPolygon, .adjustTestTO, adjustTestOT, adjustTestTZ, adjustZT
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="142">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -368,6 +368,9 @@
     <t xml:space="preserve">targets for 101</t>
   </si>
   <si>
+    <t xml:space="preserve">TT</t>
+  </si>
+  <si>
     <t xml:space="preserve">horAngle</t>
   </si>
   <si>
@@ -426,6 +429,27 @@
   </si>
   <si>
     <t xml:space="preserve">RatioZ = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:7244</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:4990</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZT</t>
   </si>
 </sst>
 </file>
@@ -851,7 +875,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.2265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1447,7 +1471,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.13671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2532,7 +2556,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2702,7 +2726,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3308,8 +3332,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:N109"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
@@ -3324,329 +3348,335 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+    </row>
+    <row r="2" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="C1" s="28" t="s">
+      <c r="B2" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="E1" s="29" t="s">
+      <c r="D2" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="E2" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="F2" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="G2" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="I1" s="29" t="s">
+      <c r="H2" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="J1" s="29" t="s">
+      <c r="I2" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J2" s="29" t="s">
         <v>107</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K2" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="L1" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="M1" s="29" t="s">
+      <c r="L2" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="N1" s="29" t="s">
+      <c r="M2" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N2" s="29" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
-        <v>1008</v>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="32" t="n">
-        <v>196534</v>
-      </c>
-      <c r="J2" s="32" t="n">
-        <v>456961430</v>
-      </c>
-      <c r="K2" s="32" t="n">
-        <v>2261163707</v>
-      </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>457619</v>
+        <v>0</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>68689</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>-11</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>6142</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>68659</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>2045</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="E3" s="32" t="n">
+        <v>196534</v>
       </c>
       <c r="J3" s="32" t="n">
-        <v>456988790</v>
+        <v>456961430</v>
       </c>
       <c r="K3" s="32" t="n">
-        <v>2261202196</v>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>-286</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <f aca="false">C3*B20</f>
-        <v>-1.52941307445672</v>
-      </c>
-      <c r="N3" s="32" t="n">
-        <v>17720</v>
-      </c>
+        <v>2261163707</v>
+      </c>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
-        <v>100</v>
+        <v>1007</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>636053</v>
+        <v>457619</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>64987</v>
+        <v>68689</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1290184</v>
+        <v>6142</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>64961</v>
+        <v>68659</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>-1832</v>
+        <v>2045</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="J4" s="1" t="n">
-        <v>457057453</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>2261204245</v>
+      <c r="J4" s="32" t="n">
+        <v>456988790</v>
+      </c>
+      <c r="K4" s="32" t="n">
+        <v>2261202196</v>
       </c>
       <c r="L4" s="1" t="n">
-        <v>-174</v>
+        <v>-286</v>
       </c>
       <c r="M4" s="1" t="n">
-        <f aca="false">C4*B20</f>
-        <v>-1.4469852155326</v>
-      </c>
-      <c r="N4" s="1" t="n">
-        <v>17429</v>
+        <f aca="false">C4*B21</f>
+        <v>-1.52941307445672</v>
+      </c>
+      <c r="N4" s="32" t="n">
+        <v>17720</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>355217</v>
+        <v>636053</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>57154</v>
+        <v>64987</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>997390</v>
+        <v>1290184</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>7018</v>
+        <v>64961</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>-56722</v>
+        <v>-1832</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>457122419</v>
+        <v>457057454</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>2261202416</v>
+        <v>2261204245</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>-928</v>
+        <v>-174</v>
       </c>
       <c r="M5" s="1" t="n">
-        <f aca="false">C5*B20</f>
-        <v>-1.27257748485928</v>
+        <f aca="false">C5*B21</f>
+        <v>-1.4469852155326</v>
       </c>
       <c r="N5" s="1" t="n">
-        <v>17255</v>
+        <v>17432</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>623634</v>
+        <v>355217</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>33730</v>
+        <v>57154</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>-11</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>973013</v>
+        <v>997390</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>166</v>
+        <v>7018</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>-33730</v>
+        <v>-56722</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="1" t="n">
-        <v>457129441</v>
+        <v>457122419</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>2261145698</v>
+        <v>2261202417</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>-560</v>
+        <v>-928</v>
       </c>
       <c r="M6" s="1" t="n">
-        <f aca="false">C6*B20</f>
-        <v>-0.751024225151407</v>
+        <f aca="false">C6*B21</f>
+        <v>-1.27257748485928</v>
       </c>
       <c r="N6" s="1" t="n">
-        <v>16327</v>
+        <v>17257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
-        <v>1003</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>653188</v>
+        <v>623634</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>33730</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>-11</v>
       </c>
-      <c r="E7" s="32" t="n">
-        <v>978190</v>
-      </c>
-      <c r="J7" s="32" t="n">
-        <v>457129609</v>
-      </c>
-      <c r="K7" s="32" t="n">
-        <v>2261111970</v>
-      </c>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32" t="n">
-        <v>15767</v>
+      <c r="E7" s="1" t="n">
+        <v>973013</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>166</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>-33730</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>457129441</v>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>2261145698</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>-560</v>
+      </c>
+      <c r="M7" s="1" t="n">
+        <f aca="false">C7*B21</f>
+        <v>-0.751024225151407</v>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>16328</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
-        <v>1004</v>
+        <v>1003</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>653188</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>978190</v>
       </c>
       <c r="J8" s="32" t="n">
-        <v>457131018</v>
+        <v>457129609</v>
       </c>
       <c r="K8" s="32" t="n">
-        <v>2261065036</v>
+        <v>2261111970</v>
       </c>
       <c r="L8" s="32"/>
       <c r="M8" s="32"/>
+      <c r="N8" s="32" t="n">
+        <v>15767</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
+      <c r="A9" s="1" t="n">
+        <v>1004</v>
+      </c>
+      <c r="J9" s="32" t="n">
+        <v>457131018</v>
+      </c>
+      <c r="K9" s="32" t="n">
+        <v>2261065036</v>
+      </c>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <f aca="false">SUM(B3:B7)</f>
-        <v>2725711</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <f aca="false">SUM(F3:F6)</f>
-        <v>140804</v>
-      </c>
-      <c r="H10" s="1" t="n">
-        <f aca="false">SUM(H3:H6)</f>
-        <v>-90239</v>
-      </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
-      <c r="L10" s="1" t="n">
-        <f aca="false">SUM(L3:L6)</f>
-        <v>-1948</v>
-      </c>
+      <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="33" t="s">
         <v>124</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>55</v>
+        <f aca="false">SUM(B4:B8)</f>
+        <v>2725711</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <f aca="false">SUM(F4:F7)</f>
+        <v>140804</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <f aca="false">SUM(H4:H7)</f>
+        <v>-90239</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
+      <c r="L11" s="1" t="n">
+        <f aca="false">SUM(L4:L7)</f>
+        <v>-1948</v>
+      </c>
       <c r="M11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3654,7 +3684,7 @@
         <v>125</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-11</v>
+        <v>55</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -3666,17 +3696,20 @@
         <v>126</v>
       </c>
       <c r="B13" s="1" t="n">
-        <f aca="false">J3+F10-J7</f>
-        <v>-15</v>
-      </c>
+        <v>-11</v>
+      </c>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B14" s="1" t="n">
-        <f aca="false">K3+H10-K7</f>
-        <v>-13</v>
+        <f aca="false">J4+F11-J8</f>
+        <v>-15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3684,7 +3717,8 @@
         <v>128</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>224560</v>
+        <f aca="false">K4+H11-K8</f>
+        <v>-13</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3692,24 +3726,23 @@
         <v>129</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>20</v>
+        <v>224560</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="1" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <f aca="false">N3+L10-N7</f>
-        <v>5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3717,8 +3750,1138 @@
         <v>133</v>
       </c>
       <c r="B20" s="1" t="n">
-        <f aca="false">B19/B15*-1</f>
+        <f aca="false">N4+L11-N8</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <f aca="false">B20/B16*-1</f>
         <v>-2.2265764161026E-005</v>
+      </c>
+    </row>
+    <row r="24" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="29"/>
+      <c r="L24" s="29"/>
+      <c r="M24" s="29"/>
+      <c r="N24" s="29"/>
+    </row>
+    <row r="25" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H25" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I25" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J25" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K25" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="L25" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="M25" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N25" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="32" t="n">
+        <v>196534</v>
+      </c>
+      <c r="J26" s="32" t="n">
+        <v>456961430</v>
+      </c>
+      <c r="K26" s="32" t="n">
+        <v>2261163707</v>
+      </c>
+      <c r="L26" s="32"/>
+      <c r="M26" s="32"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>457619</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>68689</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>68658</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>2049</v>
+      </c>
+      <c r="J27" s="32" t="n">
+        <v>456988790</v>
+      </c>
+      <c r="K27" s="32" t="n">
+        <v>2261202196</v>
+      </c>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="32" t="n">
+        <v>17720</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>64987</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>64961</v>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>-1825</v>
+      </c>
+      <c r="J28" s="1" t="n">
+        <v>457057457</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>2261204248</v>
+      </c>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1" t="n">
+        <v>17432</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>57154</v>
+      </c>
+      <c r="F29" s="1" t="n">
+        <v>7027</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>-56720</v>
+      </c>
+      <c r="J29" s="1" t="n">
+        <v>457122427</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>2261202426</v>
+      </c>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1" t="n">
+        <v>17257</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>33730</v>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>173</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>-33730</v>
+      </c>
+      <c r="J30" s="1" t="n">
+        <v>457129462</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>2261145708</v>
+      </c>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1" t="n">
+        <v>16328</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>653188</v>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="J31" s="32" t="n">
+        <v>457129639</v>
+      </c>
+      <c r="K31" s="32" t="n">
+        <v>2261111979</v>
+      </c>
+      <c r="L31" s="32"/>
+      <c r="M31" s="32"/>
+      <c r="N31" s="32" t="n">
+        <v>15767</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F33" s="1" t="n">
+        <f aca="false">SUM(F27:F30)</f>
+        <v>140819</v>
+      </c>
+      <c r="H33" s="1" t="n">
+        <f aca="false">SUM(H27:H30)</f>
+        <v>-90226</v>
+      </c>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F35" s="1" t="n">
+        <f aca="false">J27+F33-J31</f>
+        <v>-30</v>
+      </c>
+      <c r="H35" s="1" t="n">
+        <f aca="false">K27+H33-K31</f>
+        <v>-9</v>
+      </c>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="1" t="n">
+        <f aca="false">SUM(C27:C30)</f>
+        <v>224560</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="28"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="29"/>
+      <c r="L46" s="29"/>
+      <c r="M46" s="29"/>
+      <c r="N46" s="29"/>
+    </row>
+    <row r="47" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B47" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D47" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E47" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F47" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="G47" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H47" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I47" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J47" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K47" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="L47" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="M47" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N47" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>457619</v>
+      </c>
+      <c r="C48" s="1" t="n">
+        <v>68689</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>6098</v>
+      </c>
+      <c r="J48" s="32" t="n">
+        <v>456988790</v>
+      </c>
+      <c r="K48" s="32" t="n">
+        <v>2261202196</v>
+      </c>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="32" t="n">
+        <v>17720</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C49" s="1" t="n">
+        <v>64987</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>1290151</v>
+      </c>
+      <c r="J49" s="1" t="n">
+        <v>457057456</v>
+      </c>
+      <c r="K49" s="1" t="n">
+        <v>2261204238</v>
+      </c>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1" t="n">
+        <v>17432</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C50" s="1" t="n">
+        <v>57154</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>997368</v>
+      </c>
+      <c r="J50" s="1" t="n">
+        <v>457122424</v>
+      </c>
+      <c r="K50" s="1" t="n">
+        <v>2261202406</v>
+      </c>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1" t="n">
+        <v>17257</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C51" s="1" t="n">
+        <v>33730</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>973002</v>
+      </c>
+      <c r="J51" s="1" t="n">
+        <v>457129442</v>
+      </c>
+      <c r="K51" s="1" t="n">
+        <v>2261145694</v>
+      </c>
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+      <c r="N51" s="1" t="n">
+        <v>16328</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>653188</v>
+      </c>
+      <c r="E52" s="32" t="n">
+        <v>978190</v>
+      </c>
+      <c r="J52" s="32" t="n">
+        <v>457129609</v>
+      </c>
+      <c r="K52" s="32" t="n">
+        <v>2261111970</v>
+      </c>
+      <c r="L52" s="32"/>
+      <c r="M52" s="32"/>
+      <c r="N52" s="32" t="n">
+        <v>15767</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="n">
+        <v>1004</v>
+      </c>
+      <c r="J53" s="32" t="n">
+        <v>457131018</v>
+      </c>
+      <c r="K53" s="32" t="n">
+        <v>2261065036</v>
+      </c>
+      <c r="L53" s="32"/>
+      <c r="M53" s="32"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>-23</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>-39</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B60" s="1" t="n">
+        <f aca="false">SUM(C48:C51)</f>
+        <v>224560</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B64" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="68" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="28"/>
+      <c r="B68" s="28"/>
+      <c r="C68" s="28"/>
+      <c r="D68" s="29"/>
+      <c r="E68" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="F68" s="29"/>
+      <c r="G68" s="29"/>
+      <c r="H68" s="29"/>
+      <c r="I68" s="29"/>
+      <c r="J68" s="29"/>
+      <c r="K68" s="29"/>
+      <c r="L68" s="29"/>
+      <c r="M68" s="29"/>
+      <c r="N68" s="29"/>
+    </row>
+    <row r="69" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B69" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C69" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D69" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E69" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F69" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="G69" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H69" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I69" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J69" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K69" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="L69" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="M69" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N69" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B70" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>196534</v>
+      </c>
+      <c r="J70" s="32" t="n">
+        <v>456961430</v>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>2261163707</v>
+      </c>
+      <c r="L70" s="32"/>
+      <c r="M70" s="32"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B71" s="1" t="n">
+        <v>457619</v>
+      </c>
+      <c r="C71" s="1" t="n">
+        <v>68689</v>
+      </c>
+      <c r="J71" s="32" t="n">
+        <v>456988790</v>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>2261202196</v>
+      </c>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
+      <c r="N71" s="32" t="n">
+        <v>17720</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B72" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C72" s="1" t="n">
+        <v>64987</v>
+      </c>
+      <c r="J72" s="1" t="n">
+        <v>457057448</v>
+      </c>
+      <c r="K72" s="1" t="n">
+        <v>2261204245</v>
+      </c>
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
+      <c r="N72" s="1" t="n">
+        <v>17434</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B73" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C73" s="1" t="n">
+        <v>57154</v>
+      </c>
+      <c r="J73" s="1" t="n">
+        <v>457122409</v>
+      </c>
+      <c r="K73" s="1" t="n">
+        <v>2261202420</v>
+      </c>
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
+      <c r="N73" s="1" t="n">
+        <v>17260</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B74" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C74" s="1" t="n">
+        <v>33730</v>
+      </c>
+      <c r="J74" s="1" t="n">
+        <v>457129436</v>
+      </c>
+      <c r="K74" s="1" t="n">
+        <v>2261145700</v>
+      </c>
+      <c r="L74" s="1"/>
+      <c r="M74" s="1"/>
+      <c r="N74" s="1" t="n">
+        <v>16332</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E75" s="32"/>
+      <c r="J75" s="32"/>
+      <c r="K75" s="32"/>
+      <c r="L75" s="32"/>
+      <c r="M75" s="32"/>
+      <c r="N75" s="32"/>
+    </row>
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J76" s="32"/>
+      <c r="K76" s="32"/>
+      <c r="L76" s="32"/>
+      <c r="M76" s="32"/>
+    </row>
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J77" s="1"/>
+      <c r="K77" s="1"/>
+      <c r="L77" s="1"/>
+      <c r="M77" s="1"/>
+    </row>
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="B78" s="1" t="n">
+        <f aca="false">SUM(B71:B75)</f>
+        <v>2072523</v>
+      </c>
+      <c r="J78" s="1"/>
+      <c r="K78" s="1"/>
+      <c r="L78" s="1"/>
+      <c r="M78" s="1"/>
+    </row>
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B79" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" s="1"/>
+      <c r="K79" s="1"/>
+      <c r="L79" s="1"/>
+      <c r="M79" s="1"/>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J80" s="1"/>
+      <c r="K80" s="1"/>
+      <c r="L80" s="1"/>
+      <c r="M80" s="1"/>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B81" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B82" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B83" s="1" t="n">
+        <f aca="false">SUM(C71:C73)</f>
+        <v>190830</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B84" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B87" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="91" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="28"/>
+      <c r="B91" s="28"/>
+      <c r="C91" s="28"/>
+      <c r="D91" s="29"/>
+      <c r="E91" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="F91" s="29"/>
+      <c r="G91" s="29"/>
+      <c r="H91" s="29"/>
+      <c r="I91" s="29"/>
+      <c r="J91" s="29"/>
+      <c r="K91" s="29"/>
+      <c r="L91" s="29"/>
+      <c r="M91" s="29"/>
+      <c r="N91" s="29"/>
+    </row>
+    <row r="92" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B92" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C92" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D92" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E92" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F92" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="G92" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H92" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I92" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J92" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K92" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="L92" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="M92" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N92" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B93" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C93" s="1" t="n">
+        <v>64987</v>
+      </c>
+      <c r="J93" s="1" t="n">
+        <v>457057472</v>
+      </c>
+      <c r="K93" s="1" t="n">
+        <v>2261204265</v>
+      </c>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+      <c r="N93" s="1" t="n">
+        <v>17429</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B94" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C94" s="1" t="n">
+        <v>57154</v>
+      </c>
+      <c r="J94" s="1" t="n">
+        <v>457122433</v>
+      </c>
+      <c r="K94" s="1" t="n">
+        <v>2261202422</v>
+      </c>
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
+      <c r="N94" s="1" t="n">
+        <v>17255</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B95" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C95" s="1" t="n">
+        <v>33730</v>
+      </c>
+      <c r="J95" s="1" t="n">
+        <v>457129445</v>
+      </c>
+      <c r="K95" s="1" t="n">
+        <v>2261145700</v>
+      </c>
+      <c r="L95" s="1"/>
+      <c r="M95" s="1"/>
+      <c r="N95" s="1" t="n">
+        <v>16327</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B96" s="1" t="n">
+        <v>653188</v>
+      </c>
+      <c r="E96" s="32" t="n">
+        <v>978190</v>
+      </c>
+      <c r="J96" s="32" t="n">
+        <v>457129609</v>
+      </c>
+      <c r="K96" s="32" t="n">
+        <v>2261111970</v>
+      </c>
+      <c r="L96" s="32"/>
+      <c r="M96" s="32"/>
+      <c r="N96" s="32" t="n">
+        <v>15767</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="n">
+        <v>1004</v>
+      </c>
+      <c r="J97" s="32" t="n">
+        <v>457131018</v>
+      </c>
+      <c r="K97" s="32" t="n">
+        <v>2261065036</v>
+      </c>
+      <c r="L97" s="32"/>
+      <c r="M97" s="32"/>
+    </row>
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J98" s="1"/>
+      <c r="K98" s="1"/>
+      <c r="L98" s="1"/>
+      <c r="M98" s="1"/>
+    </row>
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="J99" s="1"/>
+      <c r="K99" s="1"/>
+      <c r="L99" s="1"/>
+      <c r="M99" s="1"/>
+    </row>
+    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J100" s="1"/>
+      <c r="K100" s="1"/>
+      <c r="L100" s="1"/>
+      <c r="M100" s="1"/>
+    </row>
+    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J101" s="1"/>
+      <c r="K101" s="1"/>
+      <c r="L101" s="1"/>
+      <c r="M101" s="1"/>
+    </row>
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B104" s="1" t="n">
+        <f aca="false">SUM(C93:C95)</f>
+        <v>155871</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add: PolygonCalculator.adjustPolygon, .adjustPolygonTestOO, .getPolygonRotationAngle
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="144">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -450,6 +450,12 @@
   </si>
   <si>
     <t xml:space="preserve">ZT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:2994</t>
   </si>
 </sst>
 </file>
@@ -875,7 +881,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.23828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1471,7 +1477,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2556,7 +2562,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2726,7 +2732,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3332,8 +3338,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N109"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:N130"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
@@ -4884,6 +4890,257 @@
         <v>134</v>
       </c>
     </row>
+    <row r="112" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="28"/>
+      <c r="B112" s="28"/>
+      <c r="C112" s="28"/>
+      <c r="D112" s="29"/>
+      <c r="E112" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="F112" s="29"/>
+      <c r="G112" s="29"/>
+      <c r="H112" s="29"/>
+      <c r="I112" s="29"/>
+      <c r="J112" s="29"/>
+      <c r="K112" s="29"/>
+      <c r="L112" s="29"/>
+      <c r="M112" s="29"/>
+      <c r="N112" s="29"/>
+    </row>
+    <row r="113" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="B113" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C113" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D113" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E113" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="F113" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="G113" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="H113" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I113" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="J113" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="K113" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="L113" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="M113" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="N113" s="29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C114" s="1" t="n">
+        <v>68689</v>
+      </c>
+      <c r="J114" s="32" t="n">
+        <v>456988700</v>
+      </c>
+      <c r="K114" s="32" t="n">
+        <v>2261202196</v>
+      </c>
+      <c r="L114" s="1"/>
+      <c r="M114" s="1"/>
+      <c r="N114" s="32" t="n">
+        <v>17720</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B115" s="1" t="n">
+        <v>636053</v>
+      </c>
+      <c r="C115" s="1" t="n">
+        <v>64987</v>
+      </c>
+      <c r="J115" s="1" t="n">
+        <v>457057377</v>
+      </c>
+      <c r="K115" s="1" t="n">
+        <v>2261204252</v>
+      </c>
+      <c r="L115" s="1"/>
+      <c r="M115" s="1"/>
+      <c r="N115" s="1" t="n">
+        <v>17432</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B116" s="1" t="n">
+        <v>355217</v>
+      </c>
+      <c r="C116" s="1" t="n">
+        <v>57154</v>
+      </c>
+      <c r="J116" s="1" t="n">
+        <v>457122357</v>
+      </c>
+      <c r="K116" s="1" t="n">
+        <v>2261202434</v>
+      </c>
+      <c r="L116" s="1"/>
+      <c r="M116" s="1"/>
+      <c r="N116" s="1" t="n">
+        <v>17257</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B117" s="1" t="n">
+        <v>623634</v>
+      </c>
+      <c r="C117" s="1" t="n">
+        <v>33730</v>
+      </c>
+      <c r="J117" s="1" t="n">
+        <v>457129416</v>
+      </c>
+      <c r="K117" s="1" t="n">
+        <v>2261145706</v>
+      </c>
+      <c r="L117" s="1"/>
+      <c r="M117" s="1"/>
+      <c r="N117" s="1" t="n">
+        <v>16328</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="n">
+        <v>1003</v>
+      </c>
+      <c r="E118" s="32"/>
+      <c r="J118" s="32" t="n">
+        <v>457129609</v>
+      </c>
+      <c r="K118" s="32" t="n">
+        <v>2261111970</v>
+      </c>
+      <c r="L118" s="32"/>
+      <c r="M118" s="32"/>
+      <c r="N118" s="32" t="n">
+        <v>15767</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J119" s="1"/>
+      <c r="K119" s="1"/>
+      <c r="L119" s="1"/>
+      <c r="M119" s="1"/>
+    </row>
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="J120" s="1"/>
+      <c r="K120" s="1"/>
+      <c r="L120" s="1"/>
+      <c r="M120" s="1"/>
+    </row>
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J121" s="1"/>
+      <c r="K121" s="1"/>
+      <c r="L121" s="1"/>
+      <c r="M121" s="1"/>
+    </row>
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J122" s="1"/>
+      <c r="K122" s="1"/>
+      <c r="L122" s="1"/>
+      <c r="M122" s="1"/>
+    </row>
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B123" s="1" t="n">
+        <v>-63</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B124" s="1" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B125" s="1" t="n">
+        <f aca="false">SUM(C114:C117)</f>
+        <v>224560</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B126" s="1" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B129" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Add: Extract domain creates in class diagramm. DirectCalculator.doubleToLonge, .getHorAngle, --Test
</commit_message>
<xml_diff>
--- a/project_journal.xlsx
+++ b/project_journal.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="1" state="visible" r:id="rId2"/>
@@ -13,6 +13,7 @@
     <sheet name="InverseTask test data" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Survey test data" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Polygon test data" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="DirectCalculatorTest" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="149">
   <si>
     <t xml:space="preserve">Краткое описание выполненной работы</t>
   </si>
@@ -456,6 +457,21 @@
   </si>
   <si>
     <t xml:space="preserve">1:2994</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.getHorDistance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inclinedDistance, mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TiltAngle, dms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tiltAngle, sek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horDistanse, mm</t>
   </si>
 </sst>
 </file>
@@ -881,7 +897,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E46"/>
-  <sheetFormatPr defaultColWidth="12.25390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.2734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="75.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.86"/>
@@ -1477,7 +1493,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF35"/>
-  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.71"/>
@@ -2562,7 +2578,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.5"/>
@@ -2732,7 +2748,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.82"/>
@@ -3339,16 +3355,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N130"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.16"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.65"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="21.22"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11.59"/>
   </cols>
@@ -5150,4 +5166,132 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.89"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>1.0203</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>3723</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>99984</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>-1.0203</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>-3723</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>99984</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>15.0101</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>54061</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>96585</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>